<commit_message>
docs: replace real grant numbers with virtual placeholders (66668888, 99998888777700001)
</commit_message>
<xml_diff>
--- a/assets/funding_info_template.xlsx
+++ b/assets/funding_info_template.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>62572389</t>
+          <t>66668888</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>JSGG20220831103000001</t>
+          <t>99998888777700001</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">

</xml_diff>